<commit_message>
chore: pick up local modification to superseded 08-14 density-caliber page7 workbook (not script-generated; preserved as-is)
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA/analysis/page7小结/page7_分组汇总_2026-08-14_最终.xlsx
+++ b/DATA/analysis/page7小结/page7_分组汇总_2026-08-14_最终.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\emotion_map\DATA\analysis\page7小结\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C97E050-4A2E-4A3F-9E5C-2C53D028F9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8959A4F4-CE5A-4942-AF34-3D59AA2B5655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7950" yWindow="3090" windowWidth="24135" windowHeight="17040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1原表" sheetId="1" r:id="rId1"/>
@@ -281,6 +281,7 @@
       <sz val="11"/>
       <color rgb="FF808080"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -309,6 +310,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -316,6 +318,7 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -323,6 +326,7 @@
       <sz val="11"/>
       <color rgb="FF1F4E79"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -330,6 +334,7 @@
       <sz val="11"/>
       <color rgb="FFC55A11"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -520,11 +525,47 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -537,42 +578,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -888,40 +893,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="39" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15"/>
-      <c r="F1" s="14" t="s">
+      <c r="E1" s="30"/>
+      <c r="F1" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="15"/>
-      <c r="H1" s="14" t="s">
+      <c r="G1" s="30"/>
+      <c r="H1" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="28" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
       <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
@@ -934,10 +939,10 @@
       <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
     </row>
     <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3">
@@ -1611,15 +1616,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="H1:H2"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D3:D22">
@@ -1699,15 +1704,15 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A3" s="5">
@@ -1825,15 +1830,15 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A9" s="8">
@@ -2020,15 +2025,15 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A18" s="11">
@@ -2208,7 +2213,7 @@
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="14.375" style="36" customWidth="1"/>
+    <col min="2" max="2" width="14.375" style="21" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="18.375" customWidth="1"/>
@@ -2216,22 +2221,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.15">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="14" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2246,422 +2251,422 @@
       <c r="F2" s="25"/>
     </row>
     <row r="3" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A3" s="26">
+      <c r="A3" s="15">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="15">
         <v>66</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="15">
         <v>56.1</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="15">
         <v>177.3</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A4" s="26">
+      <c r="A4" s="15">
         <v>2</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="15">
         <v>94</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="15">
         <v>30.9</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="15">
         <v>166</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A5" s="26">
+      <c r="A5" s="15">
         <v>3</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="15">
         <v>39</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="15">
         <v>43.6</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="15">
         <v>274.39999999999998</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A6" s="26">
+      <c r="A6" s="15">
         <v>4</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="15">
         <v>44</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="15">
         <v>36.4</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="15">
         <v>261.39999999999998</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A7" s="26">
+      <c r="A7" s="15">
         <v>5</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="15">
         <v>30</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="15">
         <v>30</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="15">
         <v>370</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A9" s="30">
+      <c r="A9" s="17">
         <v>6</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="30">
+      <c r="C9" s="17">
         <v>127</v>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="17">
         <v>84.3</v>
       </c>
-      <c r="E9" s="30">
+      <c r="E9" s="17">
         <v>5.5</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A10" s="30">
+      <c r="A10" s="17">
         <v>7</v>
       </c>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="17">
         <v>78</v>
       </c>
-      <c r="D10" s="30">
+      <c r="D10" s="17">
         <v>116.7</v>
       </c>
-      <c r="E10" s="30">
+      <c r="E10" s="17">
         <v>44.9</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A11" s="30">
+      <c r="A11" s="17">
         <v>8</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="17">
         <v>56</v>
       </c>
-      <c r="D11" s="30">
+      <c r="D11" s="17">
         <v>150</v>
       </c>
-      <c r="E11" s="30">
+      <c r="E11" s="17">
         <v>35.700000000000003</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A12" s="30">
+      <c r="A12" s="17">
         <v>9</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="30">
+      <c r="C12" s="17">
         <v>78</v>
       </c>
-      <c r="D12" s="30">
+      <c r="D12" s="17">
         <v>105.1</v>
       </c>
-      <c r="E12" s="30">
+      <c r="E12" s="17">
         <v>6.4</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A13" s="30">
+      <c r="A13" s="17">
         <v>10</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="30">
+      <c r="C13" s="17">
         <v>58</v>
       </c>
-      <c r="D13" s="30">
+      <c r="D13" s="17">
         <v>112.1</v>
       </c>
-      <c r="E13" s="30">
+      <c r="E13" s="17">
         <v>1.7</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A14" s="30">
+      <c r="A14" s="17">
         <v>11</v>
       </c>
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="30">
+      <c r="C14" s="17">
         <v>130</v>
       </c>
-      <c r="D14" s="30">
+      <c r="D14" s="17">
         <v>47.7</v>
       </c>
-      <c r="E14" s="30">
+      <c r="E14" s="17">
         <v>49.2</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A15" s="30">
+      <c r="A15" s="17">
         <v>12</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="30">
+      <c r="C15" s="17">
         <v>93</v>
       </c>
-      <c r="D15" s="30">
+      <c r="D15" s="17">
         <v>54.8</v>
       </c>
-      <c r="E15" s="30">
+      <c r="E15" s="17">
         <v>78.5</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A16" s="30">
+      <c r="A16" s="17">
         <v>13</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="30">
+      <c r="C16" s="17">
         <v>48</v>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="17">
         <v>77.099999999999994</v>
       </c>
-      <c r="E16" s="30">
+      <c r="E16" s="17">
         <v>0</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" x14ac:dyDescent="0.25">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
     </row>
     <row r="18" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A18" s="34">
+      <c r="A18" s="19">
         <v>14</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="19">
         <v>84</v>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="19">
         <v>13.1</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="19">
         <v>707.1</v>
       </c>
-      <c r="F18" s="35" t="s">
+      <c r="F18" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A19" s="34">
+      <c r="A19" s="19">
         <v>15</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="19">
         <v>69</v>
       </c>
-      <c r="D19" s="34">
+      <c r="D19" s="19">
         <v>10.1</v>
       </c>
-      <c r="E19" s="34">
+      <c r="E19" s="19">
         <v>726.1</v>
       </c>
-      <c r="F19" s="35" t="s">
+      <c r="F19" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A20" s="34">
+      <c r="A20" s="19">
         <v>16</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="34">
+      <c r="C20" s="19">
         <v>106</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="19">
         <v>16</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="19">
         <v>393.4</v>
       </c>
-      <c r="F20" s="35" t="s">
+      <c r="F20" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A21" s="34">
+      <c r="A21" s="19">
         <v>17</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="34">
+      <c r="C21" s="19">
         <v>66</v>
       </c>
-      <c r="D21" s="34">
+      <c r="D21" s="19">
         <v>13.6</v>
       </c>
-      <c r="E21" s="34">
+      <c r="E21" s="19">
         <v>563.6</v>
       </c>
-      <c r="F21" s="35" t="s">
+      <c r="F21" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A22" s="34">
+      <c r="A22" s="19">
         <v>18</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="34">
+      <c r="C22" s="19">
         <v>83</v>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="19">
         <v>2.4</v>
       </c>
-      <c r="E22" s="34">
+      <c r="E22" s="19">
         <v>271.10000000000002</v>
       </c>
-      <c r="F22" s="35" t="s">
+      <c r="F22" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A23" s="34">
+      <c r="A23" s="19">
         <v>19</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B23" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="34">
+      <c r="C23" s="19">
         <v>97</v>
       </c>
-      <c r="D23" s="34">
+      <c r="D23" s="19">
         <v>7.2</v>
       </c>
-      <c r="E23" s="34">
+      <c r="E23" s="19">
         <v>228.9</v>
       </c>
-      <c r="F23" s="35" t="s">
+      <c r="F23" s="20" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.5" x14ac:dyDescent="0.15">
-      <c r="A24" s="34">
+      <c r="A24" s="19">
         <v>20</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="34">
+      <c r="C24" s="19">
         <v>55</v>
       </c>
-      <c r="D24" s="34">
+      <c r="D24" s="19">
         <v>14.5</v>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="19">
         <v>401.8</v>
       </c>
-      <c r="F24" s="35" t="s">
+      <c r="F24" s="20" t="s">
         <v>61</v>
       </c>
     </row>

</xml_diff>